<commit_message>
Add login manual test cases
</commit_message>
<xml_diff>
--- a/manual-tests/Manual_Test_cases.xlsx
+++ b/manual-tests/Manual_Test_cases.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\OrangeHRM-Testing-Assignment\manual-tests\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CB1448-00FF-4437-8206-6B7F93EFEF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,13 +20,114 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>TC_MAN_001</t>
+  </si>
+  <si>
+    <t>Login with empty username and password</t>
+  </si>
+  <si>
+    <t>OrangeHRM login page is accessible</t>
+  </si>
+  <si>
+    <t>1. Leave Username empty
+2. Leave Password empty
+3. Click Login</t>
+  </si>
+  <si>
+    <t>Appropriate required-field validation messages 
+should be displayed and login should not proceed</t>
+  </si>
+  <si>
+    <t>Appropriate required-field validation messages
+ is displayed and login is not proceed</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>TC_MAN_002</t>
+  </si>
+  <si>
+    <t>Login with special characters in username and password</t>
+  </si>
+  <si>
+    <t>1. Enter special characters such as !@#$%^&amp;* in Username
+2. Enter special characters in Password
+3. Click Login</t>
+  </si>
+  <si>
+    <t>System should safely handle the input and should not crash or bypass authentication</t>
+  </si>
+  <si>
+    <t>System safely handle the input and did not crash
+ or bypass authentication</t>
+  </si>
+  <si>
+    <t>TC_MAN_003</t>
+  </si>
+  <si>
+    <t>Login with valid credentials after multiple
+ failed attempts</t>
+  </si>
+  <si>
+    <t>Valid OrangeHRM account is available</t>
+  </si>
+  <si>
+    <t>1. Enter invalid credentials and click Login several times
+2. Enter valid credentials</t>
+  </si>
+  <si>
+    <t>System should safely handle the input and should logged in successfully.</t>
+  </si>
+  <si>
+    <t>System safely handle the input and logged in successfully.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +135,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,13 +196,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +499,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.21875" customWidth="1"/>
+    <col min="2" max="2" width="38.5546875" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" customWidth="1"/>
+    <col min="4" max="4" width="42.21875" customWidth="1"/>
+    <col min="5" max="5" width="43" customWidth="1"/>
+    <col min="6" max="6" width="52.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" customWidth="1"/>
+    <col min="8" max="9" width="12.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G4" xr:uid="{95D99FB3-270C-4032-B963-DB1D393C0F18}">
+      <formula1>"Passed,Failed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:I4" xr:uid="{C996DDF9-8BB4-4A7B-89BC-EA779278EAFC}">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PIM section manual Test cases
</commit_message>
<xml_diff>
--- a/manual-tests/Manual_Test_cases.xlsx
+++ b/manual-tests/Manual_Test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\OrangeHRM-Testing-Assignment\manual-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CB1448-00FF-4437-8206-6B7F93EFEF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1B0517-C69B-4EF2-B0EB-EB60F6F3358A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="57">
   <si>
     <t>Test ID</t>
   </si>
@@ -121,13 +121,113 @@
   </si>
   <si>
     <t>System safely handle the input and logged in successfully.</t>
+  </si>
+  <si>
+    <t>TC_MAN_004</t>
+  </si>
+  <si>
+    <t>TC_MAN_005</t>
+  </si>
+  <si>
+    <t>TC_MAN_006</t>
+  </si>
+  <si>
+    <t>TC_MAN_007</t>
+  </si>
+  <si>
+    <t>TC_MAN_008</t>
+  </si>
+  <si>
+    <t>TC_MAN_009</t>
+  </si>
+  <si>
+    <t>TC_MAN_010</t>
+  </si>
+  <si>
+    <t>Verify user search with special characters</t>
+  </si>
+  <si>
+    <t>User is logged in and Admin → User Management
+ is accessible</t>
+  </si>
+  <si>
+    <t>1. Navigate to Admin → User Management. 
+2. Enter special characters such as @#$% in the 
+Username search field. 3. Click Search.</t>
+  </si>
+  <si>
+    <t>System should handle the special characters without error and display No Records Found if no
+matching  username exists.</t>
+  </si>
+  <si>
+    <t>No Records Found is displayed.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Verify all employee details fields are editable 
+when adding a new employee</t>
+  </si>
+  <si>
+    <t>User is logged in with valid Admin credentials and is on 
+PIM → Add Employee page</t>
+  </si>
+  <si>
+    <t>1. Navigate to PIM → Add Employee. 
+2. Enter data in each available Employee Details 
+field. 
+3. Try to edit/fill all fields one by one.</t>
+  </si>
+  <si>
+    <t>All applicable Employee Details fields should allow
+ the user to enter and edit data successfully.</t>
+  </si>
+  <si>
+    <t>All Employee Details fields cannot be filled successfully.</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Verify whether an existing employee record 
+can be deleted from the Employee List</t>
+  </si>
+  <si>
+    <t>User is logged in and has access to PIM → Employee List</t>
+  </si>
+  <si>
+    <t>1. Navigate to PIM → Employee List. 2. Select an existing employee record. 3. Click the Delete option. 4. Confirm the deletion if prompted.</t>
+  </si>
+  <si>
+    <t>System should prevent unauthorized or accidental deletion of an existing employee record, or require appropriate confirmation/permission before deletion.</t>
+  </si>
+  <si>
+    <t>Existing employee data can be deleted from the Employee List.</t>
+  </si>
+  <si>
+    <t>Verify update success message is displayed 
+only after completing the employee field update</t>
+  </si>
+  <si>
+    <t>1. Navigate to PIM → Employee List. 2. Select an existing employee. 3. Enter or modify a value in one employee field. 4. Without filling or modifying any other field, observe the system behavior.</t>
+  </si>
+  <si>
+    <t>Update should be completed only after the user finishes the required editing action and submits/saves the changes. A success message should be displayed only after the update is successfully saved.</t>
+  </si>
+  <si>
+    <t>Update Successful message is displayed immediately after
+ entering a value in one field, before the user completes the remaining employee fields.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,8 +268,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -186,6 +300,16 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -196,12 +320,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -218,10 +344,27 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="5">
+    <cellStyle name="Accent3" xfId="4" builtinId="37"/>
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -500,12 +643,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" customWidth="1"/>
     <col min="2" max="2" width="38.5546875" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" customWidth="1"/>
+    <col min="3" max="3" width="51.88671875" customWidth="1"/>
     <col min="4" max="4" width="42.21875" customWidth="1"/>
     <col min="5" max="5" width="43" customWidth="1"/>
     <col min="6" max="6" width="52.5546875" bestFit="1" customWidth="1"/>
@@ -629,13 +772,171 @@
         <v>16</v>
       </c>
     </row>
+    <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="78" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G4" xr:uid="{95D99FB3-270C-4032-B963-DB1D393C0F18}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G11" xr:uid="{95D99FB3-270C-4032-B963-DB1D393C0F18}">
       <formula1>"Passed,Failed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:I4" xr:uid="{C996DDF9-8BB4-4A7B-89BC-EA779278EAFC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:I11" xr:uid="{C996DDF9-8BB4-4A7B-89BC-EA779278EAFC}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Leave,Admin manual test case & Bug report
</commit_message>
<xml_diff>
--- a/manual-tests/Manual_Test_cases.xlsx
+++ b/manual-tests/Manual_Test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\OrangeHRM-Testing-Assignment\manual-tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C1B0517-C69B-4EF2-B0EB-EB60F6F3358A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8F1D1B-466A-4C1D-A015-BF4D207D3316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="85">
   <si>
     <t>Test ID</t>
   </si>
@@ -221,13 +221,138 @@
   <si>
     <t>Update Successful message is displayed immediately after
  entering a value in one field, before the user completes the remaining employee fields.</t>
+  </si>
+  <si>
+    <t>Verify Admin can successfully update a user role</t>
+  </si>
+  <si>
+    <t>Admin user is logged in and has access to Admin → 
+User Management</t>
+  </si>
+  <si>
+    <t>1. Navigate to Admin → User Management. 2. Search for an existing user. 3. Click the Edit option. 4. Change the user role. 5. Click Save. 6. Refresh the page and verify the user details.</t>
+  </si>
+  <si>
+    <t>The user role should be updated successfully, a success message should be displayed, and the updated role should persist after refreshing the page.</t>
+  </si>
+  <si>
+    <t>User role is successfully updated and the change persists after refreshing the page.</t>
+  </si>
+  <si>
+    <t>Verify that Role Filter in Admin Section works perfectly</t>
+  </si>
+  <si>
+    <t>1. Admin user is logged in successfully.
+2. Admin Panel/Section is accessible.
+3. Multiple users exist with different roles (e.g., Admin, Manager, User, Editor).
+4. Role Filter dropdown/option is available on the user list page.</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Admin Section.
+2. Go to the User List / Manage Users page.
+3. Locate the Role Filter dropdown.
+4. Select a specific role (e.g., "Admin").
+5. Click on Apply / Filter button (ifapplicable).</t>
+  </si>
+  <si>
+    <t>1. Only users matching the selected role should be displayed.
+2. User count should reflect the filtered result.
+3. Selecting "All" should display all users regardless of role.
+4. Filter should work correctly for every role option without any error.</t>
+  </si>
+  <si>
+    <t>Role Filter works perfectly — correct users are displayed based on the selected role, and "All" shows the complete user list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that after assigning leave to an employee, the leave request appears in the Approve/Reject list </t>
+  </si>
+  <si>
+    <t>1. Admin/HR user is logged in successfully.
+2. Leave Section/Module is accessible.
+3. At least one employee exists in the system.
+4. Employee has available leave balance.
+5. Leave types (e.g., Casual, Sick, Annual) are configured.
+6. Initially, the Leave List is empty (no leave requests exist).</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Leave Section.
+2. Verify that the Leave List is empty before assigning any leave.
+3. Click on Assign Leave button/option.
+4. Select an Employee from the dropdown/list.
+5. Select Leave Type (e.g., Casual Leave).
+6. Enter From Date and To Date.
+7. Add Remarks/Reason (if required).
+8. Click on Submit / Assign button.
+9. Go back to the Leave List 
+10. Verify the newly assigned leave record.</t>
+  </si>
+  <si>
+    <t>1. Before assignment, the Leave List should be empty.
+2. After assigning leave, the record should appear in the Leave List.
+3. The assigned leave should be available under Approve / Reject options.
+4. Status of the leave should be Pending (default).
+5. Employee's leave balance should be updated/reflected accordingly.
+6. No error message should be displayed.</t>
+  </si>
+  <si>
+    <t>Before assignment, the Leave List was empty. After assigning leave, the record successfully appeared in the list and is available for Approve / Reject action.</t>
+  </si>
+  <si>
+    <t>BUG REPORT</t>
+  </si>
+  <si>
+    <t>BUG_Report_1</t>
+  </si>
+  <si>
+    <t>BUG_ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Steps To Reproduce</t>
+  </si>
+  <si>
+    <t>Attachment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	PIM (Personal Information Management)</t>
+  </si>
+  <si>
+    <t>Future date cannot be selected in the Driving
+License field while adding/viewing an employee in PIM Section</t>
+  </si>
+  <si>
+    <t>1.Navigate to the PIM Section.
+2.Click on Add Employee.
+3.Fill in all initial employee details (First Name, Last Name, 4.Employee ID, etc.).
+5.Click on Save.
+6.System automatically navigates to the All Details 7.Personal Details section.
+8.Locate the Driving License field (with Date / Expiry Date).
+9.Try to select a Future Date using the date picker.
+10.Observe the behavior.</t>
+  </si>
+  <si>
+    <t>1.User (Admin/HR) is logged in successfully.
+2.PIM Section is accessible.
+3.User has permission to add a new employee.
+4.A valid Employee form is available with all required fields.</t>
+  </si>
+  <si>
+    <t>User should be able to select a Future Date in the Driving License field.</t>
+  </si>
+  <si>
+    <t>The Driving License field does not allow selecting a Future Date.</t>
+  </si>
+  <si>
+    <t>https://streamable.com/eaeo6l</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,6 +406,45 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -320,14 +484,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -338,32 +503,39 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="4" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
     <cellStyle name="Accent3" xfId="4" builtinId="37"/>
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8"/>
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -643,17 +815,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.21875" customWidth="1"/>
-    <col min="2" max="2" width="38.5546875" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="51.88671875" customWidth="1"/>
     <col min="4" max="4" width="42.21875" customWidth="1"/>
     <col min="5" max="5" width="43" customWidth="1"/>
     <col min="6" max="6" width="52.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" customWidth="1"/>
-    <col min="8" max="9" width="12.88671875" customWidth="1"/>
+    <col min="7" max="8" width="19.44140625" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -704,13 +876,13 @@
       <c r="F2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="5" t="s">
+      <c r="H2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>16</v>
       </c>
     </row>
@@ -733,13 +905,13 @@
       <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
@@ -762,71 +934,71 @@
       <c r="F4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="78" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="6" t="s">
+      <c r="H6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="8" t="s">
         <v>40</v>
       </c>
     </row>
@@ -834,7 +1006,7 @@
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -846,16 +1018,16 @@
       <c r="E7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="5" t="s">
+      <c r="H7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="7" t="s">
         <v>16</v>
       </c>
     </row>
@@ -863,7 +1035,7 @@
       <c r="A8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -875,59 +1047,173 @@
       <c r="E8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="6" t="s">
+      <c r="H8" s="8" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I8" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="78" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="6" t="s">
+      <c r="B9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="6" t="s">
+      <c r="B10" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>40</v>
+      <c r="B11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="D15" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -936,11 +1222,14 @@
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G11" xr:uid="{95D99FB3-270C-4032-B963-DB1D393C0F18}">
       <formula1>"Passed,Failed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:I11" xr:uid="{C996DDF9-8BB4-4A7B-89BC-EA779278EAFC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:I11 I18:J18" xr:uid="{C996DDF9-8BB4-4A7B-89BC-EA779278EAFC}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H18" r:id="rId1" xr:uid="{4E7F273D-BE4B-447E-AA37-7565676D502D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>